<commit_message>
case study portfolio addditions
</commit_message>
<xml_diff>
--- a/Innovatech_TCO_Comparison_2.xlsx
+++ b/Innovatech_TCO_Comparison_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\spart\Desktop\case-study-1-Innovatech\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA43322F-2947-4DFA-8E7D-7104F293A660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63CA9E31-D767-4CFF-9EF7-A8BA5D9D22EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="95">
   <si>
     <t>EC2 t3.small on-demand, $/hr</t>
   </si>
@@ -88,9 +88,6 @@
   </si>
   <si>
     <t>EBS gp3, $/GB-month</t>
-  </si>
-  <si>
-    <t>Base rate $0.08/GB-mo (us-east-1); Frankfurt storage/compute pricing runs ~15-16% higher per confirmed EC2 and NAT Gateway lookups, so that differential is applied here — recommend confirming via AWS Pricing Calculator before final submission</t>
   </si>
   <si>
     <t>EBS per web instance, GB</t>
@@ -786,12 +783,12 @@
   <sheetData>
     <row r="1" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -802,7 +799,7 @@
         <v>2.4E-2</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -813,7 +810,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -835,7 +832,7 @@
         <v>2</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -865,7 +862,7 @@
         <v>1</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -905,244 +902,244 @@
       <c r="B18" s="5">
         <v>9.2299999999999993E-2</v>
       </c>
-      <c r="C18" s="22" t="s">
-        <v>17</v>
+      <c r="C18" s="23" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" s="5">
         <v>20</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20" s="5">
         <v>100</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" s="5">
         <v>20</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B24" s="5">
         <v>5.1999999999999998E-2</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B25" s="5">
         <v>5.1999999999999998E-2</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B26" s="5">
         <v>50</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" s="5">
         <v>2.5999999999999999E-2</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B28" s="5">
         <v>9.1999999999999998E-3</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" s="5">
         <v>2</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B30" s="5">
         <v>5.7700000000000001E-2</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B31" s="5">
         <v>5</v>
       </c>
       <c r="C31" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B32" s="5">
         <v>2.3099999999999999E-2</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B33" s="5">
         <v>100</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B34" s="5">
         <v>0.05</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B35" s="5">
         <v>0.09</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B36" s="5">
         <v>30</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B39" s="6">
         <v>0.08</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B40" s="6">
         <v>0.03</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B41" s="5">
         <v>50</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B42" s="5">
         <v>4</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B43" s="5">
         <v>8</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B44" s="5">
         <v>4.33</v>
@@ -1194,6 +1191,7 @@
     <hyperlink ref="C32" r:id="rId12" xr:uid="{1E92C2DA-C953-4AA3-B979-351E54D50C57}"/>
     <hyperlink ref="C34" r:id="rId13" xr:uid="{763198B2-206A-40BE-9D82-023DFC94A799}"/>
     <hyperlink ref="C35" r:id="rId14" xr:uid="{56863F20-7FC3-4FA4-B194-11B2DD86C3CF}"/>
+    <hyperlink ref="C18" r:id="rId15" xr:uid="{7438BA0D-63C2-43F1-A7F3-D5D533E22A5B}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1212,31 +1210,31 @@
   <sheetData>
     <row r="1" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="7" t="s">
         <v>49</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>52</v>
       </c>
       <c r="C5" s="8">
         <f>Assumptions!$B$9*Assumptions!$B$10*Assumptions!$B$6*Assumptions!$B$8</f>
@@ -1245,10 +1243,10 @@
     </row>
     <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C6" s="11">
         <f>Assumptions!$B$12*Assumptions!$B$7*Assumptions!$B$8</f>
@@ -1257,10 +1255,10 @@
     </row>
     <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C7" s="8">
         <f>Assumptions!$B$14*Assumptions!$B$6*Assumptions!$B$8</f>
@@ -1269,10 +1267,10 @@
     </row>
     <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C8" s="11">
         <f>Assumptions!$B$9*Assumptions!$B$19*Assumptions!$B$18</f>
@@ -1281,10 +1279,10 @@
     </row>
     <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C9" s="8">
         <f>Assumptions!$B$12*Assumptions!$B$20*Assumptions!$B$18</f>
@@ -1293,10 +1291,10 @@
     </row>
     <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C10" s="11">
         <f>Assumptions!$B$14*Assumptions!$B$21*Assumptions!$B$18</f>
@@ -1305,10 +1303,10 @@
     </row>
     <row r="11" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C11" s="8">
         <f>Assumptions!$B$24*Assumptions!$B$8</f>
@@ -1317,10 +1315,10 @@
     </row>
     <row r="12" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C12" s="11">
         <f>Assumptions!$B$25*Assumptions!$B$26</f>
@@ -1329,10 +1327,10 @@
     </row>
     <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C13" s="8">
         <f>Assumptions!$B$27*Assumptions!$B$8</f>
@@ -1341,10 +1339,10 @@
     </row>
     <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C14" s="11">
         <f>Assumptions!$B$28*Assumptions!$B$29*Assumptions!$B$8</f>
@@ -1353,10 +1351,10 @@
     </row>
     <row r="15" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C15" s="8">
         <f>Assumptions!$B$30*Assumptions!$B$31*Assumptions!$B$8</f>
@@ -1365,10 +1363,10 @@
     </row>
     <row r="16" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C16" s="11">
         <f>Assumptions!$B$32*Assumptions!$B$33</f>
@@ -1377,10 +1375,10 @@
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C17" s="8">
         <f>Assumptions!$B$34*Assumptions!$B$8</f>
@@ -1389,10 +1387,10 @@
     </row>
     <row r="18" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C18" s="11">
         <f>Assumptions!$B$35*Assumptions!$B$36</f>
@@ -1401,7 +1399,7 @@
     </row>
     <row r="19" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="14">
@@ -1411,7 +1409,7 @@
     </row>
     <row r="21" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C21" s="8">
         <f>Assumptions!$B$42*Assumptions!$B$44*Assumptions!$B$41</f>
@@ -1420,7 +1418,7 @@
     </row>
     <row r="22" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C22" s="15">
         <v>0</v>
@@ -1428,7 +1426,7 @@
     </row>
     <row r="23" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B23" s="13"/>
       <c r="C23" s="14">
@@ -1438,21 +1436,21 @@
     </row>
     <row r="25" spans="1:4" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B25" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="C25" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="D25" s="7" t="s">
         <v>72</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B26" s="15">
         <f>C19*12</f>
@@ -1469,7 +1467,7 @@
     </row>
     <row r="27" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B27" s="16">
         <f>B26*(1+Assumptions!$B$39)</f>
@@ -1486,7 +1484,7 @@
     </row>
     <row r="28" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B28" s="15">
         <f>B27*(1+Assumptions!$B$39)</f>
@@ -1503,7 +1501,7 @@
     </row>
     <row r="29" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B29" s="16">
         <f>B28*(1+Assumptions!$B$39)</f>
@@ -1520,7 +1518,7 @@
     </row>
     <row r="30" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B30" s="15">
         <f>B29*(1+Assumptions!$B$39)</f>
@@ -1537,7 +1535,7 @@
     </row>
     <row r="31" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B31" s="18"/>
       <c r="C31" s="18"/>
@@ -1548,7 +1546,7 @@
     </row>
     <row r="32" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B32" s="18"/>
       <c r="C32" s="18"/>

</xml_diff>